<commit_message>
feat: consolida geração mensal do livro ponto por professor
</commit_message>
<xml_diff>
--- a/modelos/Modelo_de_Ponto_Mensal_Instrutor.xlsx
+++ b/modelos/Modelo_de_Ponto_Mensal_Instrutor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b898349cc0e2bfac/EMCA/Prestação de Contas FAPETI/202609 - Setembro/Planilhas das Aulas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\LivroPontoEMCA\modelos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="605" documentId="13_ncr:1_{DEA50E7C-8687-4154-856E-8E080ADC853C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2626990-625D-4B55-AC79-6C0C8021B01D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F53C1641-CAAA-4AC1-A8F0-843FEF81FA4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="754" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="754" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="192">
   <si>
     <t>Mês/Ano:</t>
   </si>
@@ -611,6 +611,12 @@
   </si>
   <si>
     <t>Noturno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assum Feres Junior </t>
+  </si>
+  <si>
+    <t>Instrutor Especialista em Gestão de Qualidade</t>
   </si>
 </sst>
 </file>
@@ -620,7 +626,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mmmm/yyyy"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -657,6 +663,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -683,7 +697,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -776,26 +790,185 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
+      <left style="medium">
+        <color indexed="64"/>
       </left>
-      <right/>
-      <top/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FF000000"/>
       </left>
       <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -805,21 +978,21 @@
         <color rgb="FF000000"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
+      <bottom style="medium">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -827,8 +1000,66 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="medium">
         <color indexed="64"/>
@@ -840,192 +1071,15 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -1034,7 +1088,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1062,99 +1116,114 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2485,81 +2554,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
     </row>
     <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
     </row>
     <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="38" t="str">
+      <c r="B3" s="22" t="str">
         <f>Base!B2</f>
         <v>CELSO FERREIRA DOS SANTOS</v>
       </c>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="38"/>
-      <c r="J3" s="38"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="39">
+      <c r="B4" s="35">
         <f>Base!E2</f>
         <v>46266</v>
       </c>
-      <c r="C4" s="39"/>
+      <c r="C4" s="35"/>
       <c r="D4" s="1"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="33"/>
-      <c r="J4" s="33"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="28" t="str">
+      <c r="B5" s="30" t="str">
         <f>Base!C2</f>
         <v>INS, SEL</v>
       </c>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
       <c r="H5" s="1" t="s">
         <v>2</v>
       </c>
@@ -2581,10 +2650,10 @@
       <c r="D7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="40" t="s">
+      <c r="E7" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="41"/>
+      <c r="F7" s="34"/>
       <c r="G7" s="6" t="s">
         <v>9</v>
       </c>
@@ -3059,36 +3128,36 @@
       <c r="J29" s="3"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F34" s="31" t="s">
+      <c r="F34" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="G34" s="31"/>
-      <c r="H34" s="31"/>
-      <c r="I34" s="31"/>
-      <c r="J34" s="31"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="25"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="25"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F39" s="31" t="s">
+      <c r="F39" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="G39" s="31"/>
-      <c r="H39" s="31"/>
-      <c r="I39" s="31"/>
-      <c r="J39" s="31"/>
+      <c r="G39" s="25"/>
+      <c r="H39" s="25"/>
+      <c r="I39" s="25"/>
+      <c r="J39" s="25"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="32" t="s">
+      <c r="A41" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="B41" s="33"/>
-      <c r="C41" s="33"/>
-      <c r="D41" s="33"/>
-      <c r="E41" s="33"/>
-      <c r="F41" s="33"/>
-      <c r="G41" s="33"/>
-      <c r="H41" s="33"/>
-      <c r="I41" s="33"/>
-      <c r="J41" s="33"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="28"/>
+      <c r="F41" s="28"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="28"/>
+      <c r="I41" s="28"/>
+      <c r="J41" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -3120,126 +3189,126 @@
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="14" width="7.85546875" customWidth="1"/>
+    <col min="3" max="14" width="7.140625" customWidth="1"/>
     <col min="15" max="15" width="14.5703125" customWidth="1"/>
     <col min="16" max="16" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
     </row>
     <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
-      <c r="L2" s="38"/>
-      <c r="M2" s="38"/>
-      <c r="N2" s="38"/>
-      <c r="O2" s="38"/>
-      <c r="P2" s="38"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
     </row>
     <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="38" t="str">
+      <c r="B3" s="22" t="str">
         <f>Base!B2</f>
         <v>CELSO FERREIRA DOS SANTOS</v>
       </c>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="38"/>
-      <c r="J3" s="38"/>
-      <c r="K3" s="38"/>
-      <c r="L3" s="38"/>
-      <c r="M3" s="38"/>
-      <c r="N3" s="38"/>
-      <c r="O3" s="38"/>
-      <c r="P3" s="38"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="42">
+      <c r="B4" s="32">
         <f>Base!E2</f>
         <v>46266</v>
       </c>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="42"/>
-      <c r="I4" s="42"/>
-      <c r="J4" s="42"/>
-      <c r="K4" s="33"/>
-      <c r="L4" s="33"/>
-      <c r="M4" s="33"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="33"/>
-      <c r="P4" s="33"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="28"/>
+      <c r="N4" s="28"/>
+      <c r="O4" s="28"/>
+      <c r="P4" s="28"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="38" t="str">
+      <c r="B5" s="22" t="str">
         <f>Base!C2</f>
         <v>INS, SEL</v>
       </c>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="38"/>
-      <c r="I5" s="38"/>
-      <c r="J5" s="38"/>
-      <c r="K5" s="38"/>
-      <c r="L5" s="38"/>
-      <c r="M5" s="38"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
       <c r="N5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="O5" s="38" t="str">
+      <c r="O5" s="22" t="str">
         <f>Base!D2</f>
         <v>CEL 26</v>
       </c>
-      <c r="P5" s="38"/>
+      <c r="P5" s="22"/>
     </row>
     <row r="6" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -3257,636 +3326,602 @@
       <c r="M6" s="7"/>
       <c r="N6" s="1"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C7" s="34" t="s">
+    <row r="7" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="40" t="s">
         <v>188</v>
       </c>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="34" t="s">
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="40" t="s">
         <v>189</v>
       </c>
-      <c r="J7" s="35"/>
-      <c r="K7" s="35"/>
-      <c r="L7" s="35"/>
-      <c r="M7" s="35"/>
-      <c r="N7" s="36"/>
+      <c r="J7" s="41"/>
+      <c r="K7" s="41"/>
+      <c r="L7" s="41"/>
+      <c r="M7" s="41"/>
+      <c r="N7" s="42"/>
     </row>
     <row r="8" spans="1:16" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="29" t="s">
+      <c r="E8" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="30"/>
-      <c r="G8" s="25" t="s">
+      <c r="F8" s="24"/>
+      <c r="G8" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="26" t="s">
+      <c r="H8" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="I8" s="27" t="s">
+      <c r="I8" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="J8" s="25" t="s">
+      <c r="J8" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="K8" s="29" t="s">
+      <c r="K8" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="L8" s="30"/>
-      <c r="M8" s="25" t="s">
+      <c r="L8" s="24"/>
+      <c r="M8" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="N8" s="26" t="s">
+      <c r="N8" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="O8" s="12" t="s">
+      <c r="O8" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="P8" s="6" t="s">
+      <c r="P8" s="36" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4">
+      <c r="A9" s="45">
         <v>46266</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="17"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
-      <c r="F9" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="H9" s="18" t="s">
-        <v>186</v>
-      </c>
-      <c r="I9" s="17"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="11"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
-      <c r="L9" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="M9" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="N9" s="18" t="s">
-        <v>186</v>
-      </c>
-      <c r="O9" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="P9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="37"/>
+      <c r="P9" s="37"/>
     </row>
     <row r="10" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+      <c r="A10" s="46">
         <v>46267</v>
       </c>
       <c r="B10" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="19"/>
+      <c r="C10" s="13"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
-      <c r="F10" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="H10" s="18" t="s">
-        <v>186</v>
-      </c>
-      <c r="I10" s="19"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="13"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
-      <c r="L10" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="N10" s="18" t="s">
-        <v>186</v>
-      </c>
-      <c r="O10" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="P10" s="3"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="37"/>
+      <c r="P10" s="38"/>
     </row>
     <row r="11" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+      <c r="A11" s="46">
         <v>46268</v>
       </c>
       <c r="B11" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="19"/>
+      <c r="C11" s="13"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="19"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="13"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
-      <c r="N11" s="20"/>
-      <c r="O11" s="16"/>
-      <c r="P11" s="3"/>
+      <c r="N11" s="14"/>
+      <c r="O11" s="38"/>
+      <c r="P11" s="38"/>
     </row>
     <row r="12" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+      <c r="A12" s="46">
         <v>46269</v>
       </c>
       <c r="B12" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="19"/>
+      <c r="C12" s="13"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="19"/>
+      <c r="H12" s="14"/>
+      <c r="I12" s="13"/>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
-      <c r="N12" s="20"/>
-      <c r="O12" s="16"/>
-      <c r="P12" s="3"/>
+      <c r="N12" s="14"/>
+      <c r="O12" s="38"/>
+      <c r="P12" s="38"/>
     </row>
     <row r="13" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+      <c r="A13" s="46">
         <v>46272</v>
       </c>
       <c r="B13" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="19"/>
+      <c r="C13" s="13"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="19"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="13"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
-      <c r="N13" s="20"/>
-      <c r="O13" s="16"/>
-      <c r="P13" s="3"/>
+      <c r="N13" s="14"/>
+      <c r="O13" s="38"/>
+      <c r="P13" s="38"/>
     </row>
     <row r="14" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+      <c r="A14" s="46">
         <v>46273</v>
       </c>
       <c r="B14" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>104</v>
-      </c>
+      <c r="C14" s="13"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>104</v>
-      </c>
+      <c r="H14" s="14"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
-      <c r="N14" s="20"/>
-      <c r="O14" s="16" t="s">
-        <v>187</v>
-      </c>
-      <c r="P14" s="3"/>
+      <c r="N14" s="14"/>
+      <c r="O14" s="38"/>
+      <c r="P14" s="38"/>
     </row>
     <row r="15" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+      <c r="A15" s="46">
         <v>46274</v>
       </c>
       <c r="B15" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="19"/>
+      <c r="C15" s="13"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="19"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="13"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
-      <c r="N15" s="20"/>
-      <c r="O15" s="16"/>
-      <c r="P15" s="3"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="38"/>
+      <c r="P15" s="38"/>
     </row>
     <row r="16" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+      <c r="A16" s="46">
         <v>46275</v>
       </c>
       <c r="B16" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="19"/>
+      <c r="C16" s="13"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="19"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="13"/>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
-      <c r="N16" s="20"/>
-      <c r="O16" s="16"/>
-      <c r="P16" s="3"/>
+      <c r="N16" s="14"/>
+      <c r="O16" s="38"/>
+      <c r="P16" s="38"/>
     </row>
     <row r="17" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+      <c r="A17" s="46">
         <v>46276</v>
       </c>
       <c r="B17" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="19"/>
+      <c r="C17" s="13"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
-      <c r="H17" s="20"/>
-      <c r="I17" s="19"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="13"/>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
-      <c r="N17" s="20"/>
-      <c r="O17" s="16"/>
-      <c r="P17" s="3"/>
+      <c r="N17" s="14"/>
+      <c r="O17" s="38"/>
+      <c r="P17" s="38"/>
     </row>
     <row r="18" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+      <c r="A18" s="46">
         <v>46279</v>
       </c>
       <c r="B18" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="19"/>
+      <c r="C18" s="13"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="19"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="13"/>
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
-      <c r="N18" s="20"/>
-      <c r="O18" s="16"/>
-      <c r="P18" s="3"/>
+      <c r="N18" s="14"/>
+      <c r="O18" s="38"/>
+      <c r="P18" s="38"/>
     </row>
     <row r="19" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+      <c r="A19" s="46">
         <v>46280</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="19"/>
+      <c r="C19" s="13"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="19"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="13"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
-      <c r="N19" s="20"/>
-      <c r="O19" s="16"/>
-      <c r="P19" s="3"/>
+      <c r="N19" s="14"/>
+      <c r="O19" s="38"/>
+      <c r="P19" s="38"/>
     </row>
     <row r="20" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+      <c r="A20" s="46">
         <v>46281</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="19"/>
+      <c r="C20" s="13"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="19"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="13"/>
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
-      <c r="N20" s="20"/>
-      <c r="O20" s="16"/>
-      <c r="P20" s="3"/>
+      <c r="N20" s="14"/>
+      <c r="O20" s="38"/>
+      <c r="P20" s="38"/>
     </row>
     <row r="21" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+      <c r="A21" s="46">
         <v>46282</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="19"/>
+      <c r="C21" s="13"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="19"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="13"/>
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
-      <c r="N21" s="20"/>
-      <c r="O21" s="16"/>
-      <c r="P21" s="3"/>
+      <c r="N21" s="14"/>
+      <c r="O21" s="38"/>
+      <c r="P21" s="38"/>
     </row>
     <row r="22" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+      <c r="A22" s="46">
         <v>46283</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C22" s="19"/>
+      <c r="C22" s="13"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="19"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="13"/>
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
-      <c r="N22" s="20"/>
-      <c r="O22" s="16"/>
-      <c r="P22" s="3"/>
+      <c r="N22" s="14"/>
+      <c r="O22" s="38"/>
+      <c r="P22" s="38"/>
     </row>
     <row r="23" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+      <c r="A23" s="46">
         <v>46286</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C23" s="19"/>
+      <c r="C23" s="13"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="19"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="13"/>
       <c r="J23" s="3"/>
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
       <c r="M23" s="3"/>
-      <c r="N23" s="20"/>
-      <c r="O23" s="16"/>
-      <c r="P23" s="3"/>
+      <c r="N23" s="14"/>
+      <c r="O23" s="38"/>
+      <c r="P23" s="38"/>
     </row>
     <row r="24" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
+      <c r="A24" s="46">
         <v>46287</v>
       </c>
       <c r="B24" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="19"/>
+      <c r="C24" s="13"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="19"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="13"/>
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
-      <c r="N24" s="20"/>
-      <c r="O24" s="16"/>
-      <c r="P24" s="3"/>
+      <c r="N24" s="14"/>
+      <c r="O24" s="38"/>
+      <c r="P24" s="38"/>
     </row>
     <row r="25" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
+      <c r="A25" s="46">
         <v>46288</v>
       </c>
       <c r="B25" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C25" s="19"/>
+      <c r="C25" s="13"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
-      <c r="H25" s="20"/>
-      <c r="I25" s="19"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="13"/>
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
-      <c r="N25" s="20"/>
-      <c r="O25" s="16"/>
-      <c r="P25" s="3"/>
+      <c r="N25" s="14"/>
+      <c r="O25" s="38"/>
+      <c r="P25" s="38"/>
     </row>
     <row r="26" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
+      <c r="A26" s="46">
         <v>46289</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="19"/>
+      <c r="C26" s="13"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="19"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="13"/>
       <c r="J26" s="3"/>
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
-      <c r="N26" s="20"/>
-      <c r="O26" s="16"/>
-      <c r="P26" s="3"/>
+      <c r="N26" s="14"/>
+      <c r="O26" s="38"/>
+      <c r="P26" s="38"/>
     </row>
     <row r="27" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
+      <c r="A27" s="46">
         <v>46290</v>
       </c>
       <c r="B27" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="19"/>
+      <c r="C27" s="13"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
-      <c r="H27" s="20"/>
-      <c r="I27" s="19"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="13"/>
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
-      <c r="N27" s="20"/>
-      <c r="O27" s="16"/>
-      <c r="P27" s="3"/>
+      <c r="N27" s="14"/>
+      <c r="O27" s="38"/>
+      <c r="P27" s="38"/>
     </row>
     <row r="28" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
+      <c r="A28" s="46">
         <v>46293</v>
       </c>
       <c r="B28" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="19"/>
+      <c r="C28" s="13"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="19"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="13"/>
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
-      <c r="N28" s="20"/>
-      <c r="O28" s="16"/>
-      <c r="P28" s="3"/>
+      <c r="N28" s="14"/>
+      <c r="O28" s="38"/>
+      <c r="P28" s="38"/>
     </row>
     <row r="29" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
+      <c r="A29" s="46">
         <v>46294</v>
       </c>
       <c r="B29" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="19"/>
+      <c r="C29" s="13"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
-      <c r="H29" s="20"/>
-      <c r="I29" s="19"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="13"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
       <c r="M29" s="3"/>
-      <c r="N29" s="20"/>
-      <c r="O29" s="16"/>
-      <c r="P29" s="3"/>
+      <c r="N29" s="14"/>
+      <c r="O29" s="38"/>
+      <c r="P29" s="38"/>
     </row>
     <row r="30" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="2">
+      <c r="A30" s="47">
         <v>46295</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B30" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C30" s="21"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="23"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="22"/>
-      <c r="K30" s="22"/>
-      <c r="L30" s="22"/>
-      <c r="M30" s="22"/>
-      <c r="N30" s="23"/>
-      <c r="O30" s="16"/>
-      <c r="P30" s="3"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="15"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="16"/>
+      <c r="M30" s="16"/>
+      <c r="N30" s="17"/>
+      <c r="O30" s="39"/>
+      <c r="P30" s="39"/>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L35" s="31" t="s">
+      <c r="L35" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="M35" s="31"/>
-      <c r="N35" s="31"/>
-      <c r="O35" s="31"/>
-      <c r="P35" s="31"/>
+      <c r="M35" s="25"/>
+      <c r="N35" s="25"/>
+      <c r="O35" s="25"/>
+      <c r="P35" s="25"/>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M39" s="29" t="s">
+        <v>190</v>
+      </c>
+      <c r="N39" s="29"/>
+      <c r="O39" s="29"/>
+      <c r="P39" s="29"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L40" s="31" t="s">
-        <v>17</v>
-      </c>
-      <c r="M40" s="31"/>
-      <c r="N40" s="31"/>
-      <c r="O40" s="31"/>
-      <c r="P40" s="31"/>
+      <c r="L40" s="26" t="s">
+        <v>191</v>
+      </c>
+      <c r="M40" s="25"/>
+      <c r="N40" s="25"/>
+      <c r="O40" s="25"/>
+      <c r="P40" s="25"/>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A42" s="32" t="s">
+      <c r="A42" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="B42" s="33"/>
-      <c r="C42" s="33"/>
-      <c r="D42" s="33"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="33"/>
-      <c r="G42" s="33"/>
-      <c r="H42" s="33"/>
-      <c r="I42" s="33"/>
-      <c r="J42" s="33"/>
-      <c r="K42" s="33"/>
-      <c r="L42" s="33"/>
-      <c r="M42" s="33"/>
-      <c r="N42" s="33"/>
-      <c r="O42" s="33"/>
-      <c r="P42" s="33"/>
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="28"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="28"/>
+      <c r="I42" s="28"/>
+      <c r="J42" s="28"/>
+      <c r="K42" s="28"/>
+      <c r="L42" s="28"/>
+      <c r="M42" s="28"/>
+      <c r="N42" s="28"/>
+      <c r="O42" s="28"/>
+      <c r="P42" s="28"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="O1:P1"/>
     <mergeCell ref="B2:P2"/>
     <mergeCell ref="B3:P3"/>
@@ -3902,6 +3937,7 @@
     <mergeCell ref="C7:H7"/>
     <mergeCell ref="I7:N7"/>
     <mergeCell ref="O5:P5"/>
+    <mergeCell ref="M39:P39"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" scale="59" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: identifica segundo instrutor no livro ponto
</commit_message>
<xml_diff>
--- a/modelos/Modelo_de_Ponto_Mensal_Instrutor.xlsx
+++ b/modelos/Modelo_de_Ponto_Mensal_Instrutor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\LivroPontoEMCA\modelos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F53C1641-CAAA-4AC1-A8F0-843FEF81FA4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93293E02-EBA0-4DB5-B6FE-602E092CECBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="754" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="193">
   <si>
     <t>Mês/Ano:</t>
   </si>
@@ -617,6 +617,9 @@
   </si>
   <si>
     <t>Instrutor Especialista em Gestão de Qualidade</t>
+  </si>
+  <si>
+    <t>* Segundo instrutor na atividade prática conforme RBAC 141.63 (c).</t>
   </si>
 </sst>
 </file>
@@ -1149,9 +1152,46 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1167,62 +1207,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2554,81 +2557,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
     </row>
     <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
     </row>
     <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="22" t="str">
+      <c r="B3" s="32" t="str">
         <f>Base!B2</f>
         <v>CELSO FERREIRA DOS SANTOS</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="35">
+      <c r="B4" s="45">
         <f>Base!E2</f>
         <v>46266</v>
       </c>
-      <c r="C4" s="35"/>
+      <c r="C4" s="45"/>
       <c r="D4" s="1"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="33"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="30" t="str">
+      <c r="B5" s="31" t="str">
         <f>Base!C2</f>
         <v>INS, SEL</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
       <c r="H5" s="1" t="s">
         <v>2</v>
       </c>
@@ -2650,10 +2653,10 @@
       <c r="D7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="33" t="s">
+      <c r="E7" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="34"/>
+      <c r="F7" s="47"/>
       <c r="G7" s="6" t="s">
         <v>9</v>
       </c>
@@ -3128,50 +3131,50 @@
       <c r="J29" s="3"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F34" s="25" t="s">
+      <c r="F34" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="G34" s="25"/>
-      <c r="H34" s="25"/>
-      <c r="I34" s="25"/>
-      <c r="J34" s="25"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
+      <c r="I34" s="38"/>
+      <c r="J34" s="38"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F39" s="25" t="s">
+      <c r="F39" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="G39" s="25"/>
-      <c r="H39" s="25"/>
-      <c r="I39" s="25"/>
-      <c r="J39" s="25"/>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="38"/>
+      <c r="J39" s="38"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="27" t="s">
+      <c r="A41" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="B41" s="28"/>
-      <c r="C41" s="28"/>
-      <c r="D41" s="28"/>
-      <c r="E41" s="28"/>
-      <c r="F41" s="28"/>
-      <c r="G41" s="28"/>
-      <c r="H41" s="28"/>
-      <c r="I41" s="28"/>
-      <c r="J41" s="28"/>
+      <c r="B41" s="33"/>
+      <c r="C41" s="33"/>
+      <c r="D41" s="33"/>
+      <c r="E41" s="33"/>
+      <c r="F41" s="33"/>
+      <c r="G41" s="33"/>
+      <c r="H41" s="33"/>
+      <c r="I41" s="33"/>
+      <c r="J41" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A41:J41"/>
-    <mergeCell ref="E4:J4"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:G5"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="F34:J34"/>
     <mergeCell ref="F39:J39"/>
     <mergeCell ref="B3:J3"/>
     <mergeCell ref="I1:J1"/>
+    <mergeCell ref="A41:J41"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:G5"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" scale="67" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -3195,120 +3198,120 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
-      <c r="N1" s="31"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
     </row>
     <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
     </row>
     <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="22" t="str">
+      <c r="B3" s="32" t="str">
         <f>Base!B2</f>
         <v>CELSO FERREIRA DOS SANTOS</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="32"/>
+      <c r="M3" s="32"/>
+      <c r="N3" s="32"/>
+      <c r="O3" s="32"/>
+      <c r="P3" s="32"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="32">
+      <c r="B4" s="35">
         <f>Base!E2</f>
         <v>46266</v>
       </c>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="28"/>
-      <c r="M4" s="28"/>
-      <c r="N4" s="28"/>
-      <c r="O4" s="28"/>
-      <c r="P4" s="28"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="33"/>
+      <c r="L4" s="33"/>
+      <c r="M4" s="33"/>
+      <c r="N4" s="33"/>
+      <c r="O4" s="33"/>
+      <c r="P4" s="33"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="22" t="str">
+      <c r="B5" s="32" t="str">
         <f>Base!C2</f>
         <v>INS, SEL</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="32"/>
       <c r="N5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="O5" s="22" t="str">
+      <c r="O5" s="32" t="str">
         <f>Base!D2</f>
         <v>CEL 26</v>
       </c>
-      <c r="P5" s="22"/>
+      <c r="P5" s="32"/>
     </row>
     <row r="6" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -3327,28 +3330,28 @@
       <c r="N6" s="1"/>
     </row>
     <row r="7" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="40" t="s">
+      <c r="C7" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="D7" s="41"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
-      <c r="I7" s="40" t="s">
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="J7" s="41"/>
-      <c r="K7" s="41"/>
-      <c r="L7" s="41"/>
-      <c r="M7" s="41"/>
-      <c r="N7" s="42"/>
+      <c r="J7" s="42"/>
+      <c r="K7" s="42"/>
+      <c r="L7" s="42"/>
+      <c r="M7" s="42"/>
+      <c r="N7" s="43"/>
     </row>
     <row r="8" spans="1:16" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="27" t="s">
         <v>5</v>
       </c>
       <c r="C8" s="18" t="s">
@@ -3357,10 +3360,10 @@
       <c r="D8" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="23" t="s">
+      <c r="E8" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="24"/>
+      <c r="F8" s="37"/>
       <c r="G8" s="19" t="s">
         <v>9</v>
       </c>
@@ -3373,25 +3376,25 @@
       <c r="J8" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="K8" s="23" t="s">
+      <c r="K8" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="L8" s="24"/>
+      <c r="L8" s="37"/>
       <c r="M8" s="19" t="s">
         <v>9</v>
       </c>
       <c r="N8" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="O8" s="36" t="s">
+      <c r="O8" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="P8" s="36" t="s">
+      <c r="P8" s="22" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="45">
+      <c r="A9" s="28">
         <v>46266</v>
       </c>
       <c r="B9" s="12" t="s">
@@ -3409,11 +3412,11 @@
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
       <c r="N9" s="12"/>
-      <c r="O9" s="37"/>
-      <c r="P9" s="37"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="23"/>
     </row>
     <row r="10" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="46">
+      <c r="A10" s="29">
         <v>46267</v>
       </c>
       <c r="B10" s="14" t="s">
@@ -3431,11 +3434,11 @@
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
       <c r="N10" s="12"/>
-      <c r="O10" s="37"/>
-      <c r="P10" s="38"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="24"/>
     </row>
     <row r="11" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="46">
+      <c r="A11" s="29">
         <v>46268</v>
       </c>
       <c r="B11" s="14" t="s">
@@ -3453,11 +3456,11 @@
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
       <c r="N11" s="14"/>
-      <c r="O11" s="38"/>
-      <c r="P11" s="38"/>
+      <c r="O11" s="24"/>
+      <c r="P11" s="24"/>
     </row>
     <row r="12" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="46">
+      <c r="A12" s="29">
         <v>46269</v>
       </c>
       <c r="B12" s="14" t="s">
@@ -3475,11 +3478,11 @@
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
       <c r="N12" s="14"/>
-      <c r="O12" s="38"/>
-      <c r="P12" s="38"/>
+      <c r="O12" s="24"/>
+      <c r="P12" s="24"/>
     </row>
     <row r="13" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="46">
+      <c r="A13" s="29">
         <v>46272</v>
       </c>
       <c r="B13" s="14" t="s">
@@ -3497,11 +3500,11 @@
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
       <c r="N13" s="14"/>
-      <c r="O13" s="38"/>
-      <c r="P13" s="38"/>
+      <c r="O13" s="24"/>
+      <c r="P13" s="24"/>
     </row>
     <row r="14" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="46">
+      <c r="A14" s="29">
         <v>46273</v>
       </c>
       <c r="B14" s="14" t="s">
@@ -3519,11 +3522,11 @@
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="14"/>
-      <c r="O14" s="38"/>
-      <c r="P14" s="38"/>
+      <c r="O14" s="24"/>
+      <c r="P14" s="24"/>
     </row>
     <row r="15" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="46">
+      <c r="A15" s="29">
         <v>46274</v>
       </c>
       <c r="B15" s="14" t="s">
@@ -3541,11 +3544,11 @@
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="14"/>
-      <c r="O15" s="38"/>
-      <c r="P15" s="38"/>
+      <c r="O15" s="24"/>
+      <c r="P15" s="24"/>
     </row>
     <row r="16" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="46">
+      <c r="A16" s="29">
         <v>46275</v>
       </c>
       <c r="B16" s="14" t="s">
@@ -3563,11 +3566,11 @@
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
       <c r="N16" s="14"/>
-      <c r="O16" s="38"/>
-      <c r="P16" s="38"/>
+      <c r="O16" s="24"/>
+      <c r="P16" s="24"/>
     </row>
     <row r="17" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="46">
+      <c r="A17" s="29">
         <v>46276</v>
       </c>
       <c r="B17" s="14" t="s">
@@ -3585,11 +3588,11 @@
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
       <c r="N17" s="14"/>
-      <c r="O17" s="38"/>
-      <c r="P17" s="38"/>
+      <c r="O17" s="24"/>
+      <c r="P17" s="24"/>
     </row>
     <row r="18" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="46">
+      <c r="A18" s="29">
         <v>46279</v>
       </c>
       <c r="B18" s="14" t="s">
@@ -3607,11 +3610,11 @@
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
       <c r="N18" s="14"/>
-      <c r="O18" s="38"/>
-      <c r="P18" s="38"/>
+      <c r="O18" s="24"/>
+      <c r="P18" s="24"/>
     </row>
     <row r="19" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="46">
+      <c r="A19" s="29">
         <v>46280</v>
       </c>
       <c r="B19" s="14" t="s">
@@ -3629,11 +3632,11 @@
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
       <c r="N19" s="14"/>
-      <c r="O19" s="38"/>
-      <c r="P19" s="38"/>
+      <c r="O19" s="24"/>
+      <c r="P19" s="24"/>
     </row>
     <row r="20" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="46">
+      <c r="A20" s="29">
         <v>46281</v>
       </c>
       <c r="B20" s="14" t="s">
@@ -3651,11 +3654,11 @@
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
       <c r="N20" s="14"/>
-      <c r="O20" s="38"/>
-      <c r="P20" s="38"/>
+      <c r="O20" s="24"/>
+      <c r="P20" s="24"/>
     </row>
     <row r="21" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="46">
+      <c r="A21" s="29">
         <v>46282</v>
       </c>
       <c r="B21" s="14" t="s">
@@ -3673,11 +3676,11 @@
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
       <c r="N21" s="14"/>
-      <c r="O21" s="38"/>
-      <c r="P21" s="38"/>
+      <c r="O21" s="24"/>
+      <c r="P21" s="24"/>
     </row>
     <row r="22" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="46">
+      <c r="A22" s="29">
         <v>46283</v>
       </c>
       <c r="B22" s="14" t="s">
@@ -3695,11 +3698,11 @@
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
       <c r="N22" s="14"/>
-      <c r="O22" s="38"/>
-      <c r="P22" s="38"/>
+      <c r="O22" s="24"/>
+      <c r="P22" s="24"/>
     </row>
     <row r="23" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="46">
+      <c r="A23" s="29">
         <v>46286</v>
       </c>
       <c r="B23" s="14" t="s">
@@ -3717,11 +3720,11 @@
       <c r="L23" s="3"/>
       <c r="M23" s="3"/>
       <c r="N23" s="14"/>
-      <c r="O23" s="38"/>
-      <c r="P23" s="38"/>
+      <c r="O23" s="24"/>
+      <c r="P23" s="24"/>
     </row>
     <row r="24" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="46">
+      <c r="A24" s="29">
         <v>46287</v>
       </c>
       <c r="B24" s="14" t="s">
@@ -3739,11 +3742,11 @@
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
       <c r="N24" s="14"/>
-      <c r="O24" s="38"/>
-      <c r="P24" s="38"/>
+      <c r="O24" s="24"/>
+      <c r="P24" s="24"/>
     </row>
     <row r="25" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="46">
+      <c r="A25" s="29">
         <v>46288</v>
       </c>
       <c r="B25" s="14" t="s">
@@ -3761,11 +3764,11 @@
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
       <c r="N25" s="14"/>
-      <c r="O25" s="38"/>
-      <c r="P25" s="38"/>
+      <c r="O25" s="24"/>
+      <c r="P25" s="24"/>
     </row>
     <row r="26" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="46">
+      <c r="A26" s="29">
         <v>46289</v>
       </c>
       <c r="B26" s="14" t="s">
@@ -3783,11 +3786,11 @@
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
       <c r="N26" s="14"/>
-      <c r="O26" s="38"/>
-      <c r="P26" s="38"/>
+      <c r="O26" s="24"/>
+      <c r="P26" s="24"/>
     </row>
     <row r="27" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="46">
+      <c r="A27" s="29">
         <v>46290</v>
       </c>
       <c r="B27" s="14" t="s">
@@ -3805,11 +3808,11 @@
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
       <c r="N27" s="14"/>
-      <c r="O27" s="38"/>
-      <c r="P27" s="38"/>
+      <c r="O27" s="24"/>
+      <c r="P27" s="24"/>
     </row>
     <row r="28" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="46">
+      <c r="A28" s="29">
         <v>46293</v>
       </c>
       <c r="B28" s="14" t="s">
@@ -3827,11 +3830,11 @@
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
       <c r="N28" s="14"/>
-      <c r="O28" s="38"/>
-      <c r="P28" s="38"/>
+      <c r="O28" s="24"/>
+      <c r="P28" s="24"/>
     </row>
     <row r="29" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="46">
+      <c r="A29" s="29">
         <v>46294</v>
       </c>
       <c r="B29" s="14" t="s">
@@ -3849,11 +3852,11 @@
       <c r="L29" s="3"/>
       <c r="M29" s="3"/>
       <c r="N29" s="14"/>
-      <c r="O29" s="38"/>
-      <c r="P29" s="38"/>
+      <c r="O29" s="24"/>
+      <c r="P29" s="24"/>
     </row>
     <row r="30" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="47">
+      <c r="A30" s="30">
         <v>46295</v>
       </c>
       <c r="B30" s="17" t="s">
@@ -3871,63 +3874,77 @@
       <c r="L30" s="16"/>
       <c r="M30" s="16"/>
       <c r="N30" s="17"/>
-      <c r="O30" s="39"/>
-      <c r="P30" s="39"/>
+      <c r="O30" s="25"/>
+      <c r="P30" s="25"/>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="32"/>
+      <c r="K32" s="32"/>
+      <c r="L32" s="32"/>
+      <c r="M32" s="32"/>
+      <c r="N32" s="32"/>
+      <c r="O32" s="32"/>
+      <c r="P32" s="32"/>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L35" s="25" t="s">
+      <c r="L35" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="M35" s="25"/>
-      <c r="N35" s="25"/>
-      <c r="O35" s="25"/>
-      <c r="P35" s="25"/>
+      <c r="M35" s="38"/>
+      <c r="N35" s="38"/>
+      <c r="O35" s="38"/>
+      <c r="P35" s="38"/>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="M39" s="29" t="s">
+      <c r="M39" s="44" t="s">
         <v>190</v>
       </c>
-      <c r="N39" s="29"/>
-      <c r="O39" s="29"/>
-      <c r="P39" s="29"/>
+      <c r="N39" s="44"/>
+      <c r="O39" s="44"/>
+      <c r="P39" s="44"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L40" s="26" t="s">
+      <c r="L40" s="39" t="s">
         <v>191</v>
       </c>
-      <c r="M40" s="25"/>
-      <c r="N40" s="25"/>
-      <c r="O40" s="25"/>
-      <c r="P40" s="25"/>
+      <c r="M40" s="38"/>
+      <c r="N40" s="38"/>
+      <c r="O40" s="38"/>
+      <c r="P40" s="38"/>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A42" s="27" t="s">
+      <c r="A42" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="B42" s="28"/>
-      <c r="C42" s="28"/>
-      <c r="D42" s="28"/>
-      <c r="E42" s="28"/>
-      <c r="F42" s="28"/>
-      <c r="G42" s="28"/>
-      <c r="H42" s="28"/>
-      <c r="I42" s="28"/>
-      <c r="J42" s="28"/>
-      <c r="K42" s="28"/>
-      <c r="L42" s="28"/>
-      <c r="M42" s="28"/>
-      <c r="N42" s="28"/>
-      <c r="O42" s="28"/>
-      <c r="P42" s="28"/>
+      <c r="B42" s="33"/>
+      <c r="C42" s="33"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="33"/>
+      <c r="G42" s="33"/>
+      <c r="H42" s="33"/>
+      <c r="I42" s="33"/>
+      <c r="J42" s="33"/>
+      <c r="K42" s="33"/>
+      <c r="L42" s="33"/>
+      <c r="M42" s="33"/>
+      <c r="N42" s="33"/>
+      <c r="O42" s="33"/>
+      <c r="P42" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="O1:P1"/>
-    <mergeCell ref="B2:P2"/>
-    <mergeCell ref="B3:P3"/>
-    <mergeCell ref="K4:P4"/>
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="B4:J4"/>
+  <mergeCells count="17">
     <mergeCell ref="B5:M5"/>
     <mergeCell ref="K8:L8"/>
     <mergeCell ref="L35:P35"/>
@@ -3938,6 +3955,13 @@
     <mergeCell ref="I7:N7"/>
     <mergeCell ref="O5:P5"/>
     <mergeCell ref="M39:P39"/>
+    <mergeCell ref="A32:P32"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="B2:P2"/>
+    <mergeCell ref="B3:P3"/>
+    <mergeCell ref="K4:P4"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="B4:J4"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" scale="59" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>